<commit_message>
test(npu): add same-device T5 QKV baseline and execution screenshots
</commit_message>
<xml_diff>
--- a/task_submission/2.1 精度自验证报告.xlsx
+++ b/task_submission/2.1 精度自验证报告.xlsx
@@ -735,6 +735,38 @@
 </x:styleSheet>
 </file>
 
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>39</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="11430000" cy="7143750"/>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="1" name="b9454405-2330-4aa9-a147-c28b601ed678"/>
+        <xdr:cNvPicPr>
+          <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="Rf0fec601a47f4179"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+</xdr:wsDr>
+</file>
+
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office">
   <a:themeElements>
@@ -978,13 +1010,15 @@
   </x:cols>
   <x:sheetData>
     <x:row r="1" customHeight="1">
-      <x:c r="A1" s="11" t="str">
-        <x:v>精度测试总结：T5 QKV 拆分与缓存追加，2026-10-29
+      <x:c r="A1" s="11" t="inlineStr">
+        <x:is>
+          <x:t>精度测试总结：T5 QKV 拆分与缓存追加，2026-10-29
 1、Ascend910_9382 / CANN 9.1.0；开发环境，指定 OS/驱动待复测。
 2、计划/适用 35，位级一致通过 35，失败 0，未测 0（含 9 个 audit）。
 3、覆盖 FP16/BF16、空缓存、奇数维度、边界和原始位模式。
 4、shape 列为 [B,H,L,D]；完整输入/输出形状、属性及逐项结果见“完整统计”。
-5、截图待补；真实原始输出见 2.2 日志，报告不代表正式验收通过。</x:v>
+5、真实截图见D40（本次补测）；真实原始输出见 2.2 日志，报告不代表正式验收通过。</x:t>
+        </x:is>
       </x:c>
       <x:c r="B1" s="3"/>
       <x:c r="C1" s="3"/>
@@ -1025,8 +1059,10 @@
       <x:c r="C4" s="14" t="str">
         <x:v>通过</x:v>
       </x:c>
-      <x:c r="D4" t="str" s="12">
-        <x:v>缺现场截图；原始日志见本包</x:v>
+      <x:c r="D4" s="12" t="inlineStr">
+        <x:is>
+          <x:t>真实终端截图见D40；逐case详见原始日志</x:t>
+        </x:is>
       </x:c>
       <x:c r="E4" t="str" s="12">
         <x:v>T5SplitQkvAppendCache_000_float16_random</x:v>
@@ -1042,8 +1078,10 @@
       <x:c r="C5" s="14" t="str">
         <x:v>通过</x:v>
       </x:c>
-      <x:c r="D5" t="str" s="12">
-        <x:v>缺现场截图；原始日志见本包</x:v>
+      <x:c r="D5" s="12" t="inlineStr">
+        <x:is>
+          <x:t>真实终端截图见D40；逐case详见原始日志</x:t>
+        </x:is>
       </x:c>
       <x:c r="E5" t="str" s="12">
         <x:v>T5SplitQkvAppendCache_001_float16_random</x:v>
@@ -1059,8 +1097,10 @@
       <x:c r="C6" s="14" t="str">
         <x:v>通过</x:v>
       </x:c>
-      <x:c r="D6" t="str" s="12">
-        <x:v>缺现场截图；原始日志见本包</x:v>
+      <x:c r="D6" s="12" t="inlineStr">
+        <x:is>
+          <x:t>真实终端截图见D40；逐case详见原始日志</x:t>
+        </x:is>
       </x:c>
       <x:c r="E6" t="str" s="12">
         <x:v>T5SplitQkvAppendCache_002_float16_random</x:v>
@@ -1076,8 +1116,10 @@
       <x:c r="C7" s="14" t="str">
         <x:v>通过</x:v>
       </x:c>
-      <x:c r="D7" t="str" s="12">
-        <x:v>缺现场截图；原始日志见本包</x:v>
+      <x:c r="D7" s="12" t="inlineStr">
+        <x:is>
+          <x:t>真实终端截图见D40；逐case详见原始日志</x:t>
+        </x:is>
       </x:c>
       <x:c r="E7" t="str" s="12">
         <x:v>T5SplitQkvAppendCache_003_float16_random</x:v>
@@ -1093,8 +1135,10 @@
       <x:c r="C8" s="14" t="str">
         <x:v>通过</x:v>
       </x:c>
-      <x:c r="D8" t="str" s="12">
-        <x:v>缺现场截图；原始日志见本包</x:v>
+      <x:c r="D8" s="12" t="inlineStr">
+        <x:is>
+          <x:t>真实终端截图见D40；逐case详见原始日志</x:t>
+        </x:is>
       </x:c>
       <x:c r="E8" t="str" s="12">
         <x:v>T5SplitQkvAppendCache_004_float16_random</x:v>
@@ -1110,8 +1154,10 @@
       <x:c r="C9" s="14" t="str">
         <x:v>通过</x:v>
       </x:c>
-      <x:c r="D9" t="str" s="12">
-        <x:v>缺现场截图；原始日志见本包</x:v>
+      <x:c r="D9" s="12" t="inlineStr">
+        <x:is>
+          <x:t>真实终端截图见D40；逐case详见原始日志</x:t>
+        </x:is>
       </x:c>
       <x:c r="E9" t="str" s="12">
         <x:v>T5SplitQkvAppendCache_005_float16_random</x:v>
@@ -1127,8 +1173,10 @@
       <x:c r="C10" s="14" t="str">
         <x:v>通过</x:v>
       </x:c>
-      <x:c r="D10" t="str" s="12">
-        <x:v>缺现场截图；原始日志见本包</x:v>
+      <x:c r="D10" s="12" t="inlineStr">
+        <x:is>
+          <x:t>真实终端截图见D40；逐case详见原始日志</x:t>
+        </x:is>
       </x:c>
       <x:c r="E10" t="str" s="12">
         <x:v>T5SplitQkvAppendCache_006_float16_random</x:v>
@@ -1144,8 +1192,10 @@
       <x:c r="C11" s="14" t="str">
         <x:v>通过</x:v>
       </x:c>
-      <x:c r="D11" t="str" s="12">
-        <x:v>缺现场截图；原始日志见本包</x:v>
+      <x:c r="D11" s="12" t="inlineStr">
+        <x:is>
+          <x:t>真实终端截图见D40；逐case详见原始日志</x:t>
+        </x:is>
       </x:c>
       <x:c r="E11" t="str" s="12">
         <x:v>T5SplitQkvAppendCache_007_float16_random</x:v>
@@ -1161,8 +1211,10 @@
       <x:c r="C12" s="14" t="str">
         <x:v>通过</x:v>
       </x:c>
-      <x:c r="D12" t="str" s="12">
-        <x:v>缺现场截图；原始日志见本包</x:v>
+      <x:c r="D12" s="12" t="inlineStr">
+        <x:is>
+          <x:t>真实终端截图见D40；逐case详见原始日志</x:t>
+        </x:is>
       </x:c>
       <x:c r="E12" s="15" t="str">
         <x:v>T5SplitQkvAppendCache_008_float16_random</x:v>
@@ -1178,8 +1230,10 @@
       <x:c r="C13" s="14" t="str">
         <x:v>通过</x:v>
       </x:c>
-      <x:c r="D13" t="str" s="12">
-        <x:v>缺现场截图；原始日志见本包</x:v>
+      <x:c r="D13" s="12" t="inlineStr">
+        <x:is>
+          <x:t>真实终端截图见D40；逐case详见原始日志</x:t>
+        </x:is>
       </x:c>
       <x:c r="E13" t="str" s="12">
         <x:v>T5SplitQkvAppendCache_009_float16_bits</x:v>
@@ -1195,8 +1249,10 @@
       <x:c r="C14" s="14" t="str">
         <x:v>通过</x:v>
       </x:c>
-      <x:c r="D14" t="str" s="12">
-        <x:v>缺现场截图；原始日志见本包</x:v>
+      <x:c r="D14" s="12" t="inlineStr">
+        <x:is>
+          <x:t>真实终端截图见D40；逐case详见原始日志</x:t>
+        </x:is>
       </x:c>
       <x:c r="E14" t="str" s="12">
         <x:v>T5SplitQkvAppendCache_010_bfloat16_random</x:v>
@@ -1212,8 +1268,10 @@
       <x:c r="C15" s="14" t="str">
         <x:v>通过</x:v>
       </x:c>
-      <x:c r="D15" t="str" s="12">
-        <x:v>缺现场截图；原始日志见本包</x:v>
+      <x:c r="D15" s="12" t="inlineStr">
+        <x:is>
+          <x:t>真实终端截图见D40；逐case详见原始日志</x:t>
+        </x:is>
       </x:c>
       <x:c r="E15" t="str" s="12">
         <x:v>T5SplitQkvAppendCache_011_bfloat16_random</x:v>
@@ -1229,8 +1287,10 @@
       <x:c r="C16" s="14" t="str">
         <x:v>通过</x:v>
       </x:c>
-      <x:c r="D16" t="str" s="12">
-        <x:v>缺现场截图；原始日志见本包</x:v>
+      <x:c r="D16" s="12" t="inlineStr">
+        <x:is>
+          <x:t>真实终端截图见D40；逐case详见原始日志</x:t>
+        </x:is>
       </x:c>
       <x:c r="E16" t="str" s="12">
         <x:v>T5SplitQkvAppendCache_012_bfloat16_random</x:v>
@@ -1246,8 +1306,10 @@
       <x:c r="C17" s="14" t="str">
         <x:v>通过</x:v>
       </x:c>
-      <x:c r="D17" t="str" s="12">
-        <x:v>缺现场截图；原始日志见本包</x:v>
+      <x:c r="D17" s="12" t="inlineStr">
+        <x:is>
+          <x:t>真实终端截图见D40；逐case详见原始日志</x:t>
+        </x:is>
       </x:c>
       <x:c r="E17" t="str" s="12">
         <x:v>T5SplitQkvAppendCache_013_bfloat16_random</x:v>
@@ -1263,8 +1325,10 @@
       <x:c r="C18" s="14" t="str">
         <x:v>通过</x:v>
       </x:c>
-      <x:c r="D18" t="str" s="12">
-        <x:v>缺现场截图；原始日志见本包</x:v>
+      <x:c r="D18" s="12" t="inlineStr">
+        <x:is>
+          <x:t>真实终端截图见D40；逐case详见原始日志</x:t>
+        </x:is>
       </x:c>
       <x:c r="E18" t="str" s="12">
         <x:v>T5SplitQkvAppendCache_014_bfloat16_random</x:v>
@@ -1280,8 +1344,10 @@
       <x:c r="C19" s="14" t="str">
         <x:v>通过</x:v>
       </x:c>
-      <x:c r="D19" t="str" s="12">
-        <x:v>缺现场截图；原始日志见本包</x:v>
+      <x:c r="D19" s="12" t="inlineStr">
+        <x:is>
+          <x:t>真实终端截图见D40；逐case详见原始日志</x:t>
+        </x:is>
       </x:c>
       <x:c r="E19" t="str" s="12">
         <x:v>T5SplitQkvAppendCache_015_bfloat16_random</x:v>
@@ -1297,8 +1363,10 @@
       <x:c r="C20" s="14" t="str">
         <x:v>通过</x:v>
       </x:c>
-      <x:c r="D20" t="str" s="12">
-        <x:v>缺现场截图；原始日志见本包</x:v>
+      <x:c r="D20" s="12" t="inlineStr">
+        <x:is>
+          <x:t>真实终端截图见D40；逐case详见原始日志</x:t>
+        </x:is>
       </x:c>
       <x:c r="E20" t="str" s="12">
         <x:v>T5SplitQkvAppendCache_016_bfloat16_random</x:v>
@@ -1314,8 +1382,10 @@
       <x:c r="C21" s="14" t="str">
         <x:v>通过</x:v>
       </x:c>
-      <x:c r="D21" t="str" s="12">
-        <x:v>缺现场截图；原始日志见本包</x:v>
+      <x:c r="D21" s="12" t="inlineStr">
+        <x:is>
+          <x:t>真实终端截图见D40；逐case详见原始日志</x:t>
+        </x:is>
       </x:c>
       <x:c r="E21" t="str" s="12">
         <x:v>T5SplitQkvAppendCache_017_bfloat16_random</x:v>
@@ -1331,8 +1401,10 @@
       <x:c r="C22" s="14" t="str">
         <x:v>通过</x:v>
       </x:c>
-      <x:c r="D22" t="str" s="12">
-        <x:v>缺现场截图；原始日志见本包</x:v>
+      <x:c r="D22" s="12" t="inlineStr">
+        <x:is>
+          <x:t>真实终端截图见D40；逐case详见原始日志</x:t>
+        </x:is>
       </x:c>
       <x:c r="E22" t="str" s="12">
         <x:v>T5SplitQkvAppendCache_018_bfloat16_random</x:v>
@@ -1348,8 +1420,10 @@
       <x:c r="C23" s="14" t="str">
         <x:v>通过</x:v>
       </x:c>
-      <x:c r="D23" t="str" s="12">
-        <x:v>缺现场截图；原始日志见本包</x:v>
+      <x:c r="D23" s="12" t="inlineStr">
+        <x:is>
+          <x:t>真实终端截图见D40；逐case详见原始日志</x:t>
+        </x:is>
       </x:c>
       <x:c r="E23" t="str" s="12">
         <x:v>T5SplitQkvAppendCache_019_bfloat16_bits</x:v>
@@ -1365,8 +1439,10 @@
       <x:c r="C24" s="14" t="str">
         <x:v>通过</x:v>
       </x:c>
-      <x:c r="D24" t="str" s="12">
-        <x:v>缺现场截图；原始日志见本包</x:v>
+      <x:c r="D24" s="12" t="inlineStr">
+        <x:is>
+          <x:t>真实终端截图见D40；逐case详见原始日志</x:t>
+        </x:is>
       </x:c>
       <x:c r="E24" t="str" s="12">
         <x:v>T5SplitQkvAppendCache_020_float16_boundary</x:v>
@@ -1382,8 +1458,10 @@
       <x:c r="C25" s="14" t="str">
         <x:v>通过</x:v>
       </x:c>
-      <x:c r="D25" t="str" s="12">
-        <x:v>缺现场截图；原始日志见本包</x:v>
+      <x:c r="D25" s="12" t="inlineStr">
+        <x:is>
+          <x:t>真实终端截图见D40；逐case详见原始日志</x:t>
+        </x:is>
       </x:c>
       <x:c r="E25" t="str" s="12">
         <x:v>T5SplitQkvAppendCache_021_float16_boundary</x:v>
@@ -1399,8 +1477,10 @@
       <x:c r="C26" s="14" t="str">
         <x:v>通过</x:v>
       </x:c>
-      <x:c r="D26" t="str" s="12">
-        <x:v>缺现场截图；原始日志见本包</x:v>
+      <x:c r="D26" s="12" t="inlineStr">
+        <x:is>
+          <x:t>真实终端截图见D40；逐case详见原始日志</x:t>
+        </x:is>
       </x:c>
       <x:c r="E26" t="str" s="12">
         <x:v>T5SplitQkvAppendCache_022_float16_boundary</x:v>
@@ -1416,8 +1496,10 @@
       <x:c r="C27" s="14" t="str">
         <x:v>通过</x:v>
       </x:c>
-      <x:c r="D27" t="str" s="12">
-        <x:v>缺现场截图；原始日志见本包</x:v>
+      <x:c r="D27" s="12" t="inlineStr">
+        <x:is>
+          <x:t>真实终端截图见D40；逐case详见原始日志</x:t>
+        </x:is>
       </x:c>
       <x:c r="E27" t="str" s="12">
         <x:v>T5SplitQkvAppendCache_023_bfloat16_boundary</x:v>
@@ -1433,8 +1515,10 @@
       <x:c r="C28" s="14" t="str">
         <x:v>通过</x:v>
       </x:c>
-      <x:c r="D28" t="str" s="12">
-        <x:v>缺现场截图；原始日志见本包</x:v>
+      <x:c r="D28" s="12" t="inlineStr">
+        <x:is>
+          <x:t>真实终端截图见D40；逐case详见原始日志</x:t>
+        </x:is>
       </x:c>
       <x:c r="E28" t="str" s="12">
         <x:v>T5SplitQkvAppendCache_024_bfloat16_boundary</x:v>
@@ -1450,8 +1534,10 @@
       <x:c r="C29" s="14" t="str">
         <x:v>通过</x:v>
       </x:c>
-      <x:c r="D29" t="str" s="12">
-        <x:v>缺现场截图；原始日志见本包</x:v>
+      <x:c r="D29" s="12" t="inlineStr">
+        <x:is>
+          <x:t>真实终端截图见D40；逐case详见原始日志</x:t>
+        </x:is>
       </x:c>
       <x:c r="E29" t="str" s="12">
         <x:v>T5SplitQkvAppendCache_025_bfloat16_boundary</x:v>
@@ -1467,8 +1553,10 @@
       <x:c r="C30" s="14" t="str">
         <x:v>通过</x:v>
       </x:c>
-      <x:c r="D30" t="str" s="12">
-        <x:v>缺现场截图；原始日志见本包</x:v>
+      <x:c r="D30" s="12" t="inlineStr">
+        <x:is>
+          <x:t>真实终端截图见D40；逐case详见原始日志</x:t>
+        </x:is>
       </x:c>
       <x:c r="E30" t="str" s="12">
         <x:v>T5SplitQkvAppendCache_audit_026_float16_bits</x:v>
@@ -1484,8 +1572,10 @@
       <x:c r="C31" s="14" t="str">
         <x:v>通过</x:v>
       </x:c>
-      <x:c r="D31" t="str" s="12">
-        <x:v>缺现场截图；原始日志见本包</x:v>
+      <x:c r="D31" s="12" t="inlineStr">
+        <x:is>
+          <x:t>真实终端截图见D40；逐case详见原始日志</x:t>
+        </x:is>
       </x:c>
       <x:c r="E31" t="str" s="12">
         <x:v>T5SplitQkvAppendCache_audit_027_float16_bits</x:v>
@@ -1501,8 +1591,10 @@
       <x:c r="C32" s="14" t="str">
         <x:v>通过</x:v>
       </x:c>
-      <x:c r="D32" t="str" s="12">
-        <x:v>缺现场截图；原始日志见本包</x:v>
+      <x:c r="D32" s="12" t="inlineStr">
+        <x:is>
+          <x:t>真实终端截图见D40；逐case详见原始日志</x:t>
+        </x:is>
       </x:c>
       <x:c r="E32" t="str" s="12">
         <x:v>T5SplitQkvAppendCache_audit_028_float16_bits</x:v>
@@ -1518,8 +1610,10 @@
       <x:c r="C33" s="14" t="str">
         <x:v>通过</x:v>
       </x:c>
-      <x:c r="D33" t="str" s="12">
-        <x:v>缺现场截图；原始日志见本包</x:v>
+      <x:c r="D33" s="12" t="inlineStr">
+        <x:is>
+          <x:t>真实终端截图见D40；逐case详见原始日志</x:t>
+        </x:is>
       </x:c>
       <x:c r="E33" t="str" s="12">
         <x:v>T5SplitQkvAppendCache_audit_029_float16_bits</x:v>
@@ -1535,8 +1629,10 @@
       <x:c r="C34" s="14" t="str">
         <x:v>通过</x:v>
       </x:c>
-      <x:c r="D34" t="str" s="12">
-        <x:v>缺现场截图；原始日志见本包</x:v>
+      <x:c r="D34" s="12" t="inlineStr">
+        <x:is>
+          <x:t>真实终端截图见D40；逐case详见原始日志</x:t>
+        </x:is>
       </x:c>
       <x:c r="E34" t="str" s="12">
         <x:v>T5SplitQkvAppendCache_audit_030_bfloat16_bits</x:v>
@@ -1552,8 +1648,10 @@
       <x:c r="C35" s="14" t="str">
         <x:v>通过</x:v>
       </x:c>
-      <x:c r="D35" t="str" s="12">
-        <x:v>缺现场截图；原始日志见本包</x:v>
+      <x:c r="D35" s="12" t="inlineStr">
+        <x:is>
+          <x:t>真实终端截图见D40；逐case详见原始日志</x:t>
+        </x:is>
       </x:c>
       <x:c r="E35" t="str" s="12">
         <x:v>T5SplitQkvAppendCache_audit_031_bfloat16_bits</x:v>
@@ -1569,8 +1667,10 @@
       <x:c r="C36" s="14" t="str">
         <x:v>通过</x:v>
       </x:c>
-      <x:c r="D36" t="str" s="12">
-        <x:v>缺现场截图；原始日志见本包</x:v>
+      <x:c r="D36" s="12" t="inlineStr">
+        <x:is>
+          <x:t>真实终端截图见D40；逐case详见原始日志</x:t>
+        </x:is>
       </x:c>
       <x:c r="E36" t="str" s="12">
         <x:v>T5SplitQkvAppendCache_audit_032_bfloat16_bits</x:v>
@@ -1586,8 +1686,10 @@
       <x:c r="C37" s="14" t="str">
         <x:v>通过</x:v>
       </x:c>
-      <x:c r="D37" t="str" s="12">
-        <x:v>缺现场截图；原始日志见本包</x:v>
+      <x:c r="D37" s="12" t="inlineStr">
+        <x:is>
+          <x:t>真实终端截图见D40；逐case详见原始日志</x:t>
+        </x:is>
       </x:c>
       <x:c r="E37" t="str" s="12">
         <x:v>T5SplitQkvAppendCache_audit_033_bfloat16_bits</x:v>
@@ -1603,8 +1705,10 @@
       <x:c r="C38" s="14" t="str">
         <x:v>通过</x:v>
       </x:c>
-      <x:c r="D38" t="str" s="12">
-        <x:v>缺现场截图；原始日志见本包</x:v>
+      <x:c r="D38" s="12" t="inlineStr">
+        <x:is>
+          <x:t>真实终端截图见D40；逐case详见原始日志</x:t>
+        </x:is>
       </x:c>
       <x:c r="E38" t="str" s="12">
         <x:v>T5SplitQkvAppendCache_audit_034_float16_bits</x:v>
@@ -1648,6 +1752,7 @@
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcd1648bd8de44d76"/>
 </x:worksheet>
 </file>
 

</xml_diff>

<commit_message>
docs(npu): deliver repeated passing T5 QKV validation and preserved reports
</commit_message>
<xml_diff>
--- a/task_submission/2.1 精度自验证报告.xlsx
+++ b/task_submission/2.1 精度自验证报告.xlsx
@@ -747,13 +747,13 @@
     <xdr:ext cx="11430000" cy="7143750"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="1" name="b9454405-2330-4aa9-a147-c28b601ed678"/>
+        <xdr:cNvPr id="1" name="e05dea55-cd03-4b23-9dad-33c8e18113d3"/>
         <xdr:cNvPicPr>
           <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="Rf0fec601a47f4179"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R7fe1cb9e16be43f5"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -1012,12 +1012,12 @@
     <x:row r="1" customHeight="1">
       <x:c r="A1" s="11" t="inlineStr">
         <x:is>
-          <x:t>精度测试总结：T5 QKV 拆分与缓存追加，2026-10-29
-1、Ascend910_9382 / CANN 9.1.0；开发环境，指定 OS/驱动待复测。
-2、计划/适用 35，位级一致通过 35，失败 0，未测 0（含 9 个 audit）。
-3、覆盖 FP16/BF16、空缓存、奇数维度、边界和原始位模式。
-4、shape 列为 [B,H,L,D]；完整输入/输出形状、属性及逐项结果见“完整统计”。
-5、真实截图见D40（本次补测）；真实原始输出见 2.2 日志，报告不代表正式验收通过。</x:t>
+          <x:t>精度测试总结：T5 QKV拆分与缓存追加，2026-10-30
+1、Ascend910_9382 / CANN9.1.0；当前OS/driver与指定环境不同。
+2、35/35官方case逐位一致，失败0、未测0，含9个audit。
+3、两入口交叉验证及扩展206/206通过；真实截图见D40。
+4、FP16/BF16、空缓存、奇数维度、原始位模式均覆盖。
+5、被测8ea9aff；page_size:1g；完整shape和证据见完整统计。</x:t>
         </x:is>
       </x:c>
       <x:c r="B1" s="3"/>
@@ -1056,12 +1056,14 @@
       <x:c r="B4" s="14" t="str">
         <x:v>float16</x:v>
       </x:c>
-      <x:c r="C4" s="14" t="str">
-        <x:v>通过</x:v>
+      <x:c r="C4" s="14" t="inlineStr">
+        <x:is>
+          <x:t>通过</x:t>
+        </x:is>
       </x:c>
       <x:c r="D4" s="12" t="inlineStr">
         <x:is>
-          <x:t>真实终端截图见D40；逐case详见原始日志</x:t>
+          <x:t>本次真实终端截图见D40</x:t>
         </x:is>
       </x:c>
       <x:c r="E4" t="str" s="12">
@@ -1075,12 +1077,14 @@
       <x:c r="B5" s="14" t="str">
         <x:v>float16</x:v>
       </x:c>
-      <x:c r="C5" s="14" t="str">
-        <x:v>通过</x:v>
+      <x:c r="C5" s="14" t="inlineStr">
+        <x:is>
+          <x:t>通过</x:t>
+        </x:is>
       </x:c>
       <x:c r="D5" s="12" t="inlineStr">
         <x:is>
-          <x:t>真实终端截图见D40；逐case详见原始日志</x:t>
+          <x:t>本次真实终端截图见D40</x:t>
         </x:is>
       </x:c>
       <x:c r="E5" t="str" s="12">
@@ -1094,12 +1098,14 @@
       <x:c r="B6" s="14" t="str">
         <x:v>float16</x:v>
       </x:c>
-      <x:c r="C6" s="14" t="str">
-        <x:v>通过</x:v>
+      <x:c r="C6" s="14" t="inlineStr">
+        <x:is>
+          <x:t>通过</x:t>
+        </x:is>
       </x:c>
       <x:c r="D6" s="12" t="inlineStr">
         <x:is>
-          <x:t>真实终端截图见D40；逐case详见原始日志</x:t>
+          <x:t>本次真实终端截图见D40</x:t>
         </x:is>
       </x:c>
       <x:c r="E6" t="str" s="12">
@@ -1113,12 +1119,14 @@
       <x:c r="B7" s="14" t="str">
         <x:v>float16</x:v>
       </x:c>
-      <x:c r="C7" s="14" t="str">
-        <x:v>通过</x:v>
+      <x:c r="C7" s="14" t="inlineStr">
+        <x:is>
+          <x:t>通过</x:t>
+        </x:is>
       </x:c>
       <x:c r="D7" s="12" t="inlineStr">
         <x:is>
-          <x:t>真实终端截图见D40；逐case详见原始日志</x:t>
+          <x:t>本次真实终端截图见D40</x:t>
         </x:is>
       </x:c>
       <x:c r="E7" t="str" s="12">
@@ -1132,12 +1140,14 @@
       <x:c r="B8" s="14" t="str">
         <x:v>float16</x:v>
       </x:c>
-      <x:c r="C8" s="14" t="str">
-        <x:v>通过</x:v>
+      <x:c r="C8" s="14" t="inlineStr">
+        <x:is>
+          <x:t>通过</x:t>
+        </x:is>
       </x:c>
       <x:c r="D8" s="12" t="inlineStr">
         <x:is>
-          <x:t>真实终端截图见D40；逐case详见原始日志</x:t>
+          <x:t>本次真实终端截图见D40</x:t>
         </x:is>
       </x:c>
       <x:c r="E8" t="str" s="12">
@@ -1151,12 +1161,14 @@
       <x:c r="B9" s="14" t="str">
         <x:v>float16</x:v>
       </x:c>
-      <x:c r="C9" s="14" t="str">
-        <x:v>通过</x:v>
+      <x:c r="C9" s="14" t="inlineStr">
+        <x:is>
+          <x:t>通过</x:t>
+        </x:is>
       </x:c>
       <x:c r="D9" s="12" t="inlineStr">
         <x:is>
-          <x:t>真实终端截图见D40；逐case详见原始日志</x:t>
+          <x:t>本次真实终端截图见D40</x:t>
         </x:is>
       </x:c>
       <x:c r="E9" t="str" s="12">
@@ -1170,12 +1182,14 @@
       <x:c r="B10" s="14" t="str">
         <x:v>float16</x:v>
       </x:c>
-      <x:c r="C10" s="14" t="str">
-        <x:v>通过</x:v>
+      <x:c r="C10" s="14" t="inlineStr">
+        <x:is>
+          <x:t>通过</x:t>
+        </x:is>
       </x:c>
       <x:c r="D10" s="12" t="inlineStr">
         <x:is>
-          <x:t>真实终端截图见D40；逐case详见原始日志</x:t>
+          <x:t>本次真实终端截图见D40</x:t>
         </x:is>
       </x:c>
       <x:c r="E10" t="str" s="12">
@@ -1189,12 +1203,14 @@
       <x:c r="B11" s="14" t="str">
         <x:v>float16</x:v>
       </x:c>
-      <x:c r="C11" s="14" t="str">
-        <x:v>通过</x:v>
+      <x:c r="C11" s="14" t="inlineStr">
+        <x:is>
+          <x:t>通过</x:t>
+        </x:is>
       </x:c>
       <x:c r="D11" s="12" t="inlineStr">
         <x:is>
-          <x:t>真实终端截图见D40；逐case详见原始日志</x:t>
+          <x:t>本次真实终端截图见D40</x:t>
         </x:is>
       </x:c>
       <x:c r="E11" t="str" s="12">
@@ -1208,12 +1224,14 @@
       <x:c r="B12" s="14" t="str">
         <x:v>float16</x:v>
       </x:c>
-      <x:c r="C12" s="14" t="str">
-        <x:v>通过</x:v>
+      <x:c r="C12" s="14" t="inlineStr">
+        <x:is>
+          <x:t>通过</x:t>
+        </x:is>
       </x:c>
       <x:c r="D12" s="12" t="inlineStr">
         <x:is>
-          <x:t>真实终端截图见D40；逐case详见原始日志</x:t>
+          <x:t>本次真实终端截图见D40</x:t>
         </x:is>
       </x:c>
       <x:c r="E12" s="15" t="str">
@@ -1227,12 +1245,14 @@
       <x:c r="B13" s="14" t="str">
         <x:v>float16</x:v>
       </x:c>
-      <x:c r="C13" s="14" t="str">
-        <x:v>通过</x:v>
+      <x:c r="C13" s="14" t="inlineStr">
+        <x:is>
+          <x:t>通过</x:t>
+        </x:is>
       </x:c>
       <x:c r="D13" s="12" t="inlineStr">
         <x:is>
-          <x:t>真实终端截图见D40；逐case详见原始日志</x:t>
+          <x:t>本次真实终端截图见D40</x:t>
         </x:is>
       </x:c>
       <x:c r="E13" t="str" s="12">
@@ -1246,12 +1266,14 @@
       <x:c r="B14" s="14" t="str">
         <x:v>bfloat16</x:v>
       </x:c>
-      <x:c r="C14" s="14" t="str">
-        <x:v>通过</x:v>
+      <x:c r="C14" s="14" t="inlineStr">
+        <x:is>
+          <x:t>通过</x:t>
+        </x:is>
       </x:c>
       <x:c r="D14" s="12" t="inlineStr">
         <x:is>
-          <x:t>真实终端截图见D40；逐case详见原始日志</x:t>
+          <x:t>本次真实终端截图见D40</x:t>
         </x:is>
       </x:c>
       <x:c r="E14" t="str" s="12">
@@ -1265,12 +1287,14 @@
       <x:c r="B15" s="14" t="str">
         <x:v>bfloat16</x:v>
       </x:c>
-      <x:c r="C15" s="14" t="str">
-        <x:v>通过</x:v>
+      <x:c r="C15" s="14" t="inlineStr">
+        <x:is>
+          <x:t>通过</x:t>
+        </x:is>
       </x:c>
       <x:c r="D15" s="12" t="inlineStr">
         <x:is>
-          <x:t>真实终端截图见D40；逐case详见原始日志</x:t>
+          <x:t>本次真实终端截图见D40</x:t>
         </x:is>
       </x:c>
       <x:c r="E15" t="str" s="12">
@@ -1284,12 +1308,14 @@
       <x:c r="B16" s="14" t="str">
         <x:v>bfloat16</x:v>
       </x:c>
-      <x:c r="C16" s="14" t="str">
-        <x:v>通过</x:v>
+      <x:c r="C16" s="14" t="inlineStr">
+        <x:is>
+          <x:t>通过</x:t>
+        </x:is>
       </x:c>
       <x:c r="D16" s="12" t="inlineStr">
         <x:is>
-          <x:t>真实终端截图见D40；逐case详见原始日志</x:t>
+          <x:t>本次真实终端截图见D40</x:t>
         </x:is>
       </x:c>
       <x:c r="E16" t="str" s="12">
@@ -1303,12 +1329,14 @@
       <x:c r="B17" s="14" t="str">
         <x:v>bfloat16</x:v>
       </x:c>
-      <x:c r="C17" s="14" t="str">
-        <x:v>通过</x:v>
+      <x:c r="C17" s="14" t="inlineStr">
+        <x:is>
+          <x:t>通过</x:t>
+        </x:is>
       </x:c>
       <x:c r="D17" s="12" t="inlineStr">
         <x:is>
-          <x:t>真实终端截图见D40；逐case详见原始日志</x:t>
+          <x:t>本次真实终端截图见D40</x:t>
         </x:is>
       </x:c>
       <x:c r="E17" t="str" s="12">
@@ -1322,12 +1350,14 @@
       <x:c r="B18" s="14" t="str">
         <x:v>bfloat16</x:v>
       </x:c>
-      <x:c r="C18" s="14" t="str">
-        <x:v>通过</x:v>
+      <x:c r="C18" s="14" t="inlineStr">
+        <x:is>
+          <x:t>通过</x:t>
+        </x:is>
       </x:c>
       <x:c r="D18" s="12" t="inlineStr">
         <x:is>
-          <x:t>真实终端截图见D40；逐case详见原始日志</x:t>
+          <x:t>本次真实终端截图见D40</x:t>
         </x:is>
       </x:c>
       <x:c r="E18" t="str" s="12">
@@ -1341,12 +1371,14 @@
       <x:c r="B19" s="14" t="str">
         <x:v>bfloat16</x:v>
       </x:c>
-      <x:c r="C19" s="14" t="str">
-        <x:v>通过</x:v>
+      <x:c r="C19" s="14" t="inlineStr">
+        <x:is>
+          <x:t>通过</x:t>
+        </x:is>
       </x:c>
       <x:c r="D19" s="12" t="inlineStr">
         <x:is>
-          <x:t>真实终端截图见D40；逐case详见原始日志</x:t>
+          <x:t>本次真实终端截图见D40</x:t>
         </x:is>
       </x:c>
       <x:c r="E19" t="str" s="12">
@@ -1360,12 +1392,14 @@
       <x:c r="B20" s="14" t="str">
         <x:v>bfloat16</x:v>
       </x:c>
-      <x:c r="C20" s="14" t="str">
-        <x:v>通过</x:v>
+      <x:c r="C20" s="14" t="inlineStr">
+        <x:is>
+          <x:t>通过</x:t>
+        </x:is>
       </x:c>
       <x:c r="D20" s="12" t="inlineStr">
         <x:is>
-          <x:t>真实终端截图见D40；逐case详见原始日志</x:t>
+          <x:t>本次真实终端截图见D40</x:t>
         </x:is>
       </x:c>
       <x:c r="E20" t="str" s="12">
@@ -1379,12 +1413,14 @@
       <x:c r="B21" s="14" t="str">
         <x:v>bfloat16</x:v>
       </x:c>
-      <x:c r="C21" s="14" t="str">
-        <x:v>通过</x:v>
+      <x:c r="C21" s="14" t="inlineStr">
+        <x:is>
+          <x:t>通过</x:t>
+        </x:is>
       </x:c>
       <x:c r="D21" s="12" t="inlineStr">
         <x:is>
-          <x:t>真实终端截图见D40；逐case详见原始日志</x:t>
+          <x:t>本次真实终端截图见D40</x:t>
         </x:is>
       </x:c>
       <x:c r="E21" t="str" s="12">
@@ -1398,12 +1434,14 @@
       <x:c r="B22" s="14" t="str">
         <x:v>bfloat16</x:v>
       </x:c>
-      <x:c r="C22" s="14" t="str">
-        <x:v>通过</x:v>
+      <x:c r="C22" s="14" t="inlineStr">
+        <x:is>
+          <x:t>通过</x:t>
+        </x:is>
       </x:c>
       <x:c r="D22" s="12" t="inlineStr">
         <x:is>
-          <x:t>真实终端截图见D40；逐case详见原始日志</x:t>
+          <x:t>本次真实终端截图见D40</x:t>
         </x:is>
       </x:c>
       <x:c r="E22" t="str" s="12">
@@ -1417,12 +1455,14 @@
       <x:c r="B23" s="14" t="str">
         <x:v>bfloat16</x:v>
       </x:c>
-      <x:c r="C23" s="14" t="str">
-        <x:v>通过</x:v>
+      <x:c r="C23" s="14" t="inlineStr">
+        <x:is>
+          <x:t>通过</x:t>
+        </x:is>
       </x:c>
       <x:c r="D23" s="12" t="inlineStr">
         <x:is>
-          <x:t>真实终端截图见D40；逐case详见原始日志</x:t>
+          <x:t>本次真实终端截图见D40</x:t>
         </x:is>
       </x:c>
       <x:c r="E23" t="str" s="12">
@@ -1436,12 +1476,14 @@
       <x:c r="B24" s="14" t="str">
         <x:v>float16</x:v>
       </x:c>
-      <x:c r="C24" s="14" t="str">
-        <x:v>通过</x:v>
+      <x:c r="C24" s="14" t="inlineStr">
+        <x:is>
+          <x:t>通过</x:t>
+        </x:is>
       </x:c>
       <x:c r="D24" s="12" t="inlineStr">
         <x:is>
-          <x:t>真实终端截图见D40；逐case详见原始日志</x:t>
+          <x:t>本次真实终端截图见D40</x:t>
         </x:is>
       </x:c>
       <x:c r="E24" t="str" s="12">
@@ -1455,12 +1497,14 @@
       <x:c r="B25" s="14" t="str">
         <x:v>float16</x:v>
       </x:c>
-      <x:c r="C25" s="14" t="str">
-        <x:v>通过</x:v>
+      <x:c r="C25" s="14" t="inlineStr">
+        <x:is>
+          <x:t>通过</x:t>
+        </x:is>
       </x:c>
       <x:c r="D25" s="12" t="inlineStr">
         <x:is>
-          <x:t>真实终端截图见D40；逐case详见原始日志</x:t>
+          <x:t>本次真实终端截图见D40</x:t>
         </x:is>
       </x:c>
       <x:c r="E25" t="str" s="12">
@@ -1474,12 +1518,14 @@
       <x:c r="B26" s="14" t="str">
         <x:v>float16</x:v>
       </x:c>
-      <x:c r="C26" s="14" t="str">
-        <x:v>通过</x:v>
+      <x:c r="C26" s="14" t="inlineStr">
+        <x:is>
+          <x:t>通过</x:t>
+        </x:is>
       </x:c>
       <x:c r="D26" s="12" t="inlineStr">
         <x:is>
-          <x:t>真实终端截图见D40；逐case详见原始日志</x:t>
+          <x:t>本次真实终端截图见D40</x:t>
         </x:is>
       </x:c>
       <x:c r="E26" t="str" s="12">
@@ -1493,12 +1539,14 @@
       <x:c r="B27" s="14" t="str">
         <x:v>bfloat16</x:v>
       </x:c>
-      <x:c r="C27" s="14" t="str">
-        <x:v>通过</x:v>
+      <x:c r="C27" s="14" t="inlineStr">
+        <x:is>
+          <x:t>通过</x:t>
+        </x:is>
       </x:c>
       <x:c r="D27" s="12" t="inlineStr">
         <x:is>
-          <x:t>真实终端截图见D40；逐case详见原始日志</x:t>
+          <x:t>本次真实终端截图见D40</x:t>
         </x:is>
       </x:c>
       <x:c r="E27" t="str" s="12">
@@ -1512,12 +1560,14 @@
       <x:c r="B28" s="14" t="str">
         <x:v>bfloat16</x:v>
       </x:c>
-      <x:c r="C28" s="14" t="str">
-        <x:v>通过</x:v>
+      <x:c r="C28" s="14" t="inlineStr">
+        <x:is>
+          <x:t>通过</x:t>
+        </x:is>
       </x:c>
       <x:c r="D28" s="12" t="inlineStr">
         <x:is>
-          <x:t>真实终端截图见D40；逐case详见原始日志</x:t>
+          <x:t>本次真实终端截图见D40</x:t>
         </x:is>
       </x:c>
       <x:c r="E28" t="str" s="12">
@@ -1531,12 +1581,14 @@
       <x:c r="B29" s="14" t="str">
         <x:v>bfloat16</x:v>
       </x:c>
-      <x:c r="C29" s="14" t="str">
-        <x:v>通过</x:v>
+      <x:c r="C29" s="14" t="inlineStr">
+        <x:is>
+          <x:t>通过</x:t>
+        </x:is>
       </x:c>
       <x:c r="D29" s="12" t="inlineStr">
         <x:is>
-          <x:t>真实终端截图见D40；逐case详见原始日志</x:t>
+          <x:t>本次真实终端截图见D40</x:t>
         </x:is>
       </x:c>
       <x:c r="E29" t="str" s="12">
@@ -1550,12 +1602,14 @@
       <x:c r="B30" s="14" t="str">
         <x:v>float16</x:v>
       </x:c>
-      <x:c r="C30" s="14" t="str">
-        <x:v>通过</x:v>
+      <x:c r="C30" s="14" t="inlineStr">
+        <x:is>
+          <x:t>通过</x:t>
+        </x:is>
       </x:c>
       <x:c r="D30" s="12" t="inlineStr">
         <x:is>
-          <x:t>真实终端截图见D40；逐case详见原始日志</x:t>
+          <x:t>本次真实终端截图见D40</x:t>
         </x:is>
       </x:c>
       <x:c r="E30" t="str" s="12">
@@ -1569,12 +1623,14 @@
       <x:c r="B31" s="14" t="str">
         <x:v>float16</x:v>
       </x:c>
-      <x:c r="C31" s="14" t="str">
-        <x:v>通过</x:v>
+      <x:c r="C31" s="14" t="inlineStr">
+        <x:is>
+          <x:t>通过</x:t>
+        </x:is>
       </x:c>
       <x:c r="D31" s="12" t="inlineStr">
         <x:is>
-          <x:t>真实终端截图见D40；逐case详见原始日志</x:t>
+          <x:t>本次真实终端截图见D40</x:t>
         </x:is>
       </x:c>
       <x:c r="E31" t="str" s="12">
@@ -1588,12 +1644,14 @@
       <x:c r="B32" s="14" t="str">
         <x:v>float16</x:v>
       </x:c>
-      <x:c r="C32" s="14" t="str">
-        <x:v>通过</x:v>
+      <x:c r="C32" s="14" t="inlineStr">
+        <x:is>
+          <x:t>通过</x:t>
+        </x:is>
       </x:c>
       <x:c r="D32" s="12" t="inlineStr">
         <x:is>
-          <x:t>真实终端截图见D40；逐case详见原始日志</x:t>
+          <x:t>本次真实终端截图见D40</x:t>
         </x:is>
       </x:c>
       <x:c r="E32" t="str" s="12">
@@ -1607,12 +1665,14 @@
       <x:c r="B33" s="14" t="str">
         <x:v>float16</x:v>
       </x:c>
-      <x:c r="C33" s="14" t="str">
-        <x:v>通过</x:v>
+      <x:c r="C33" s="14" t="inlineStr">
+        <x:is>
+          <x:t>通过</x:t>
+        </x:is>
       </x:c>
       <x:c r="D33" s="12" t="inlineStr">
         <x:is>
-          <x:t>真实终端截图见D40；逐case详见原始日志</x:t>
+          <x:t>本次真实终端截图见D40</x:t>
         </x:is>
       </x:c>
       <x:c r="E33" t="str" s="12">
@@ -1626,12 +1686,14 @@
       <x:c r="B34" s="14" t="str">
         <x:v>bfloat16</x:v>
       </x:c>
-      <x:c r="C34" s="14" t="str">
-        <x:v>通过</x:v>
+      <x:c r="C34" s="14" t="inlineStr">
+        <x:is>
+          <x:t>通过</x:t>
+        </x:is>
       </x:c>
       <x:c r="D34" s="12" t="inlineStr">
         <x:is>
-          <x:t>真实终端截图见D40；逐case详见原始日志</x:t>
+          <x:t>本次真实终端截图见D40</x:t>
         </x:is>
       </x:c>
       <x:c r="E34" t="str" s="12">
@@ -1645,12 +1707,14 @@
       <x:c r="B35" s="14" t="str">
         <x:v>bfloat16</x:v>
       </x:c>
-      <x:c r="C35" s="14" t="str">
-        <x:v>通过</x:v>
+      <x:c r="C35" s="14" t="inlineStr">
+        <x:is>
+          <x:t>通过</x:t>
+        </x:is>
       </x:c>
       <x:c r="D35" s="12" t="inlineStr">
         <x:is>
-          <x:t>真实终端截图见D40；逐case详见原始日志</x:t>
+          <x:t>本次真实终端截图见D40</x:t>
         </x:is>
       </x:c>
       <x:c r="E35" t="str" s="12">
@@ -1664,12 +1728,14 @@
       <x:c r="B36" s="14" t="str">
         <x:v>bfloat16</x:v>
       </x:c>
-      <x:c r="C36" s="14" t="str">
-        <x:v>通过</x:v>
+      <x:c r="C36" s="14" t="inlineStr">
+        <x:is>
+          <x:t>通过</x:t>
+        </x:is>
       </x:c>
       <x:c r="D36" s="12" t="inlineStr">
         <x:is>
-          <x:t>真实终端截图见D40；逐case详见原始日志</x:t>
+          <x:t>本次真实终端截图见D40</x:t>
         </x:is>
       </x:c>
       <x:c r="E36" t="str" s="12">
@@ -1683,12 +1749,14 @@
       <x:c r="B37" s="14" t="str">
         <x:v>bfloat16</x:v>
       </x:c>
-      <x:c r="C37" s="14" t="str">
-        <x:v>通过</x:v>
+      <x:c r="C37" s="14" t="inlineStr">
+        <x:is>
+          <x:t>通过</x:t>
+        </x:is>
       </x:c>
       <x:c r="D37" s="12" t="inlineStr">
         <x:is>
-          <x:t>真实终端截图见D40；逐case详见原始日志</x:t>
+          <x:t>本次真实终端截图见D40</x:t>
         </x:is>
       </x:c>
       <x:c r="E37" t="str" s="12">
@@ -1702,12 +1770,14 @@
       <x:c r="B38" s="14" t="str">
         <x:v>float16</x:v>
       </x:c>
-      <x:c r="C38" s="14" t="str">
-        <x:v>通过</x:v>
+      <x:c r="C38" s="14" t="inlineStr">
+        <x:is>
+          <x:t>通过</x:t>
+        </x:is>
       </x:c>
       <x:c r="D38" s="12" t="inlineStr">
         <x:is>
-          <x:t>真实终端截图见D40；逐case详见原始日志</x:t>
+          <x:t>本次真实终端截图见D40</x:t>
         </x:is>
       </x:c>
       <x:c r="E38" t="str" s="12">
@@ -1752,7 +1822,7 @@
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcd1648bd8de44d76"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2c508fc8041d4f02"/>
 </x:worksheet>
 </file>
 
@@ -1905,26 +1975,34 @@
       <x:c r="P2" s="7" t="str">
         <x:v>否</x:v>
       </x:c>
-      <x:c r="Q2" s="7" t="str">
-        <x:v>通过</x:v>
-      </x:c>
-      <x:c r="R2" s="7" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="S2" s="7" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="T2" s="7" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="U2" s="7" t="str">
-        <x:v>passed</x:v>
-      </x:c>
-      <x:c r="V2" s="7" t="str">
-        <x:v>passed</x:v>
-      </x:c>
-      <x:c r="W2" s="7" t="str">
-        <x:v>raw/reports/final_176_01/public_accuracy.json#/cases/0</x:v>
+      <x:c r="Q2" s="7" t="inlineStr">
+        <x:is>
+          <x:t>通过</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="R2" s="7">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="S2" s="7">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="T2" s="7">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="U2" s="7" t="inlineStr">
+        <x:is>
+          <x:t>passed</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="V2" s="7" t="inlineStr">
+        <x:is>
+          <x:t>passed</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="W2" s="7" t="inlineStr">
+        <x:is>
+          <x:t>raw/reports/visible_page1g_final_accuracy.json#/cases/0</x:t>
+        </x:is>
       </x:c>
     </x:row>
     <x:row r="3" ht="30" customHeight="1">
@@ -1976,26 +2054,34 @@
       <x:c r="P3" s="7" t="str">
         <x:v>否</x:v>
       </x:c>
-      <x:c r="Q3" s="7" t="str">
-        <x:v>通过</x:v>
-      </x:c>
-      <x:c r="R3" s="7" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="S3" s="7" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="T3" s="7" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="U3" s="7" t="str">
-        <x:v>passed</x:v>
-      </x:c>
-      <x:c r="V3" s="7" t="str">
-        <x:v>passed</x:v>
-      </x:c>
-      <x:c r="W3" s="7" t="str">
-        <x:v>raw/reports/final_176_01/public_accuracy.json#/cases/1</x:v>
+      <x:c r="Q3" s="7" t="inlineStr">
+        <x:is>
+          <x:t>通过</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="R3" s="7">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="S3" s="7">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="T3" s="7">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="U3" s="7" t="inlineStr">
+        <x:is>
+          <x:t>passed</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="V3" s="7" t="inlineStr">
+        <x:is>
+          <x:t>passed</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="W3" s="7" t="inlineStr">
+        <x:is>
+          <x:t>raw/reports/visible_page1g_final_accuracy.json#/cases/1</x:t>
+        </x:is>
       </x:c>
     </x:row>
     <x:row r="4" ht="30" customHeight="1">
@@ -2047,26 +2133,34 @@
       <x:c r="P4" s="7" t="str">
         <x:v>否</x:v>
       </x:c>
-      <x:c r="Q4" s="7" t="str">
-        <x:v>通过</x:v>
-      </x:c>
-      <x:c r="R4" s="7" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="S4" s="7" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="T4" s="7" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="U4" s="7" t="str">
-        <x:v>passed</x:v>
-      </x:c>
-      <x:c r="V4" s="7" t="str">
-        <x:v>passed</x:v>
-      </x:c>
-      <x:c r="W4" s="7" t="str">
-        <x:v>raw/reports/final_176_01/public_accuracy.json#/cases/2</x:v>
+      <x:c r="Q4" s="7" t="inlineStr">
+        <x:is>
+          <x:t>通过</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="R4" s="7">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="S4" s="7">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="T4" s="7">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="U4" s="7" t="inlineStr">
+        <x:is>
+          <x:t>passed</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="V4" s="7" t="inlineStr">
+        <x:is>
+          <x:t>passed</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="W4" s="7" t="inlineStr">
+        <x:is>
+          <x:t>raw/reports/visible_page1g_final_accuracy.json#/cases/2</x:t>
+        </x:is>
       </x:c>
     </x:row>
     <x:row r="5" ht="30" customHeight="1">
@@ -2118,26 +2212,34 @@
       <x:c r="P5" s="7" t="str">
         <x:v>否</x:v>
       </x:c>
-      <x:c r="Q5" s="7" t="str">
-        <x:v>通过</x:v>
-      </x:c>
-      <x:c r="R5" s="7" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="S5" s="7" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="T5" s="7" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="U5" s="7" t="str">
-        <x:v>passed</x:v>
-      </x:c>
-      <x:c r="V5" s="7" t="str">
-        <x:v>passed</x:v>
-      </x:c>
-      <x:c r="W5" s="7" t="str">
-        <x:v>raw/reports/final_176_01/public_accuracy.json#/cases/3</x:v>
+      <x:c r="Q5" s="7" t="inlineStr">
+        <x:is>
+          <x:t>通过</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="R5" s="7">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="S5" s="7">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="T5" s="7">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="U5" s="7" t="inlineStr">
+        <x:is>
+          <x:t>passed</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="V5" s="7" t="inlineStr">
+        <x:is>
+          <x:t>passed</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="W5" s="7" t="inlineStr">
+        <x:is>
+          <x:t>raw/reports/visible_page1g_final_accuracy.json#/cases/3</x:t>
+        </x:is>
       </x:c>
     </x:row>
     <x:row r="6" ht="30" customHeight="1">
@@ -2189,26 +2291,34 @@
       <x:c r="P6" s="7" t="str">
         <x:v>否</x:v>
       </x:c>
-      <x:c r="Q6" s="7" t="str">
-        <x:v>通过</x:v>
-      </x:c>
-      <x:c r="R6" s="7" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="S6" s="7" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="T6" s="7" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="U6" s="7" t="str">
-        <x:v>passed</x:v>
-      </x:c>
-      <x:c r="V6" s="7" t="str">
-        <x:v>passed</x:v>
-      </x:c>
-      <x:c r="W6" s="7" t="str">
-        <x:v>raw/reports/final_176_01/public_accuracy.json#/cases/4</x:v>
+      <x:c r="Q6" s="7" t="inlineStr">
+        <x:is>
+          <x:t>通过</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="R6" s="7">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="S6" s="7">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="T6" s="7">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="U6" s="7" t="inlineStr">
+        <x:is>
+          <x:t>passed</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="V6" s="7" t="inlineStr">
+        <x:is>
+          <x:t>passed</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="W6" s="7" t="inlineStr">
+        <x:is>
+          <x:t>raw/reports/visible_page1g_final_accuracy.json#/cases/4</x:t>
+        </x:is>
       </x:c>
     </x:row>
     <x:row r="7" ht="30" customHeight="1">
@@ -2260,26 +2370,34 @@
       <x:c r="P7" s="7" t="str">
         <x:v>否</x:v>
       </x:c>
-      <x:c r="Q7" s="7" t="str">
-        <x:v>通过</x:v>
-      </x:c>
-      <x:c r="R7" s="7" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="S7" s="7" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="T7" s="7" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="U7" s="7" t="str">
-        <x:v>passed</x:v>
-      </x:c>
-      <x:c r="V7" s="7" t="str">
-        <x:v>passed</x:v>
-      </x:c>
-      <x:c r="W7" s="7" t="str">
-        <x:v>raw/reports/final_176_01/public_accuracy.json#/cases/5</x:v>
+      <x:c r="Q7" s="7" t="inlineStr">
+        <x:is>
+          <x:t>通过</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="R7" s="7">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="S7" s="7">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="T7" s="7">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="U7" s="7" t="inlineStr">
+        <x:is>
+          <x:t>passed</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="V7" s="7" t="inlineStr">
+        <x:is>
+          <x:t>passed</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="W7" s="7" t="inlineStr">
+        <x:is>
+          <x:t>raw/reports/visible_page1g_final_accuracy.json#/cases/5</x:t>
+        </x:is>
       </x:c>
     </x:row>
     <x:row r="8" ht="30" customHeight="1">
@@ -2331,26 +2449,34 @@
       <x:c r="P8" s="7" t="str">
         <x:v>否</x:v>
       </x:c>
-      <x:c r="Q8" s="7" t="str">
-        <x:v>通过</x:v>
-      </x:c>
-      <x:c r="R8" s="7" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="S8" s="7" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="T8" s="7" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="U8" s="7" t="str">
-        <x:v>passed</x:v>
-      </x:c>
-      <x:c r="V8" s="7" t="str">
-        <x:v>passed</x:v>
-      </x:c>
-      <x:c r="W8" s="7" t="str">
-        <x:v>raw/reports/final_176_01/public_accuracy.json#/cases/6</x:v>
+      <x:c r="Q8" s="7" t="inlineStr">
+        <x:is>
+          <x:t>通过</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="R8" s="7">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="S8" s="7">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="T8" s="7">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="U8" s="7" t="inlineStr">
+        <x:is>
+          <x:t>passed</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="V8" s="7" t="inlineStr">
+        <x:is>
+          <x:t>passed</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="W8" s="7" t="inlineStr">
+        <x:is>
+          <x:t>raw/reports/visible_page1g_final_accuracy.json#/cases/6</x:t>
+        </x:is>
       </x:c>
     </x:row>
     <x:row r="9" ht="30" customHeight="1">
@@ -2402,26 +2528,34 @@
       <x:c r="P9" s="7" t="str">
         <x:v>否</x:v>
       </x:c>
-      <x:c r="Q9" s="7" t="str">
-        <x:v>通过</x:v>
-      </x:c>
-      <x:c r="R9" s="7" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="S9" s="7" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="T9" s="7" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="U9" s="7" t="str">
-        <x:v>passed</x:v>
-      </x:c>
-      <x:c r="V9" s="7" t="str">
-        <x:v>passed</x:v>
-      </x:c>
-      <x:c r="W9" s="7" t="str">
-        <x:v>raw/reports/final_176_01/public_accuracy.json#/cases/7</x:v>
+      <x:c r="Q9" s="7" t="inlineStr">
+        <x:is>
+          <x:t>通过</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="R9" s="7">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="S9" s="7">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="T9" s="7">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="U9" s="7" t="inlineStr">
+        <x:is>
+          <x:t>passed</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="V9" s="7" t="inlineStr">
+        <x:is>
+          <x:t>passed</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="W9" s="7" t="inlineStr">
+        <x:is>
+          <x:t>raw/reports/visible_page1g_final_accuracy.json#/cases/7</x:t>
+        </x:is>
       </x:c>
     </x:row>
     <x:row r="10" ht="30" customHeight="1">
@@ -2473,26 +2607,34 @@
       <x:c r="P10" s="7" t="str">
         <x:v>否</x:v>
       </x:c>
-      <x:c r="Q10" s="7" t="str">
-        <x:v>通过</x:v>
-      </x:c>
-      <x:c r="R10" s="7" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="S10" s="7" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="T10" s="7" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="U10" s="7" t="str">
-        <x:v>passed</x:v>
-      </x:c>
-      <x:c r="V10" s="7" t="str">
-        <x:v>passed</x:v>
-      </x:c>
-      <x:c r="W10" s="7" t="str">
-        <x:v>raw/reports/final_176_01/public_accuracy.json#/cases/8</x:v>
+      <x:c r="Q10" s="7" t="inlineStr">
+        <x:is>
+          <x:t>通过</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="R10" s="7">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="S10" s="7">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="T10" s="7">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="U10" s="7" t="inlineStr">
+        <x:is>
+          <x:t>passed</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="V10" s="7" t="inlineStr">
+        <x:is>
+          <x:t>passed</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="W10" s="7" t="inlineStr">
+        <x:is>
+          <x:t>raw/reports/visible_page1g_final_accuracy.json#/cases/8</x:t>
+        </x:is>
       </x:c>
     </x:row>
     <x:row r="11" ht="30" customHeight="1">
@@ -2544,26 +2686,34 @@
       <x:c r="P11" s="7" t="str">
         <x:v>否</x:v>
       </x:c>
-      <x:c r="Q11" s="7" t="str">
-        <x:v>通过</x:v>
-      </x:c>
-      <x:c r="R11" s="7" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="S11" s="7" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="T11" s="7" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="U11" s="7" t="str">
-        <x:v>passed</x:v>
-      </x:c>
-      <x:c r="V11" s="7" t="str">
-        <x:v>passed</x:v>
-      </x:c>
-      <x:c r="W11" s="7" t="str">
-        <x:v>raw/reports/final_176_01/public_accuracy.json#/cases/9</x:v>
+      <x:c r="Q11" s="7" t="inlineStr">
+        <x:is>
+          <x:t>通过</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="R11" s="7">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="S11" s="7">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="T11" s="7">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="U11" s="7" t="inlineStr">
+        <x:is>
+          <x:t>passed</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="V11" s="7" t="inlineStr">
+        <x:is>
+          <x:t>passed</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="W11" s="7" t="inlineStr">
+        <x:is>
+          <x:t>raw/reports/visible_page1g_final_accuracy.json#/cases/9</x:t>
+        </x:is>
       </x:c>
     </x:row>
     <x:row r="12" ht="30" customHeight="1">
@@ -2615,26 +2765,34 @@
       <x:c r="P12" s="7" t="str">
         <x:v>否</x:v>
       </x:c>
-      <x:c r="Q12" s="7" t="str">
-        <x:v>通过</x:v>
-      </x:c>
-      <x:c r="R12" s="7" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="S12" s="7" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="T12" s="7" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="U12" s="7" t="str">
-        <x:v>passed</x:v>
-      </x:c>
-      <x:c r="V12" s="7" t="str">
-        <x:v>passed</x:v>
-      </x:c>
-      <x:c r="W12" s="7" t="str">
-        <x:v>raw/reports/final_176_01/public_accuracy.json#/cases/10</x:v>
+      <x:c r="Q12" s="7" t="inlineStr">
+        <x:is>
+          <x:t>通过</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="R12" s="7">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="S12" s="7">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="T12" s="7">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="U12" s="7" t="inlineStr">
+        <x:is>
+          <x:t>passed</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="V12" s="7" t="inlineStr">
+        <x:is>
+          <x:t>passed</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="W12" s="7" t="inlineStr">
+        <x:is>
+          <x:t>raw/reports/visible_page1g_final_accuracy.json#/cases/10</x:t>
+        </x:is>
       </x:c>
     </x:row>
     <x:row r="13" ht="30" customHeight="1">
@@ -2686,26 +2844,34 @@
       <x:c r="P13" s="7" t="str">
         <x:v>否</x:v>
       </x:c>
-      <x:c r="Q13" s="7" t="str">
-        <x:v>通过</x:v>
-      </x:c>
-      <x:c r="R13" s="7" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="S13" s="7" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="T13" s="7" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="U13" s="7" t="str">
-        <x:v>passed</x:v>
-      </x:c>
-      <x:c r="V13" s="7" t="str">
-        <x:v>passed</x:v>
-      </x:c>
-      <x:c r="W13" s="7" t="str">
-        <x:v>raw/reports/final_176_01/public_accuracy.json#/cases/11</x:v>
+      <x:c r="Q13" s="7" t="inlineStr">
+        <x:is>
+          <x:t>通过</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="R13" s="7">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="S13" s="7">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="T13" s="7">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="U13" s="7" t="inlineStr">
+        <x:is>
+          <x:t>passed</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="V13" s="7" t="inlineStr">
+        <x:is>
+          <x:t>passed</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="W13" s="7" t="inlineStr">
+        <x:is>
+          <x:t>raw/reports/visible_page1g_final_accuracy.json#/cases/11</x:t>
+        </x:is>
       </x:c>
     </x:row>
     <x:row r="14" ht="30" customHeight="1">
@@ -2757,26 +2923,34 @@
       <x:c r="P14" s="7" t="str">
         <x:v>否</x:v>
       </x:c>
-      <x:c r="Q14" s="7" t="str">
-        <x:v>通过</x:v>
-      </x:c>
-      <x:c r="R14" s="7" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="S14" s="7" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="T14" s="7" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="U14" s="7" t="str">
-        <x:v>passed</x:v>
-      </x:c>
-      <x:c r="V14" s="7" t="str">
-        <x:v>passed</x:v>
-      </x:c>
-      <x:c r="W14" s="7" t="str">
-        <x:v>raw/reports/final_176_01/public_accuracy.json#/cases/12</x:v>
+      <x:c r="Q14" s="7" t="inlineStr">
+        <x:is>
+          <x:t>通过</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="R14" s="7">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="S14" s="7">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="T14" s="7">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="U14" s="7" t="inlineStr">
+        <x:is>
+          <x:t>passed</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="V14" s="7" t="inlineStr">
+        <x:is>
+          <x:t>passed</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="W14" s="7" t="inlineStr">
+        <x:is>
+          <x:t>raw/reports/visible_page1g_final_accuracy.json#/cases/12</x:t>
+        </x:is>
       </x:c>
     </x:row>
     <x:row r="15" ht="30" customHeight="1">
@@ -2828,26 +3002,34 @@
       <x:c r="P15" s="7" t="str">
         <x:v>否</x:v>
       </x:c>
-      <x:c r="Q15" s="7" t="str">
-        <x:v>通过</x:v>
-      </x:c>
-      <x:c r="R15" s="7" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="S15" s="7" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="T15" s="7" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="U15" s="7" t="str">
-        <x:v>passed</x:v>
-      </x:c>
-      <x:c r="V15" s="7" t="str">
-        <x:v>passed</x:v>
-      </x:c>
-      <x:c r="W15" s="7" t="str">
-        <x:v>raw/reports/final_176_01/public_accuracy.json#/cases/13</x:v>
+      <x:c r="Q15" s="7" t="inlineStr">
+        <x:is>
+          <x:t>通过</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="R15" s="7">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="S15" s="7">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="T15" s="7">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="U15" s="7" t="inlineStr">
+        <x:is>
+          <x:t>passed</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="V15" s="7" t="inlineStr">
+        <x:is>
+          <x:t>passed</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="W15" s="7" t="inlineStr">
+        <x:is>
+          <x:t>raw/reports/visible_page1g_final_accuracy.json#/cases/13</x:t>
+        </x:is>
       </x:c>
     </x:row>
     <x:row r="16" ht="30" customHeight="1">
@@ -2899,26 +3081,34 @@
       <x:c r="P16" s="7" t="str">
         <x:v>否</x:v>
       </x:c>
-      <x:c r="Q16" s="7" t="str">
-        <x:v>通过</x:v>
-      </x:c>
-      <x:c r="R16" s="7" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="S16" s="7" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="T16" s="7" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="U16" s="7" t="str">
-        <x:v>passed</x:v>
-      </x:c>
-      <x:c r="V16" s="7" t="str">
-        <x:v>passed</x:v>
-      </x:c>
-      <x:c r="W16" s="7" t="str">
-        <x:v>raw/reports/final_176_01/public_accuracy.json#/cases/14</x:v>
+      <x:c r="Q16" s="7" t="inlineStr">
+        <x:is>
+          <x:t>通过</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="R16" s="7">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="S16" s="7">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="T16" s="7">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="U16" s="7" t="inlineStr">
+        <x:is>
+          <x:t>passed</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="V16" s="7" t="inlineStr">
+        <x:is>
+          <x:t>passed</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="W16" s="7" t="inlineStr">
+        <x:is>
+          <x:t>raw/reports/visible_page1g_final_accuracy.json#/cases/14</x:t>
+        </x:is>
       </x:c>
     </x:row>
     <x:row r="17" ht="30" customHeight="1">
@@ -2970,26 +3160,34 @@
       <x:c r="P17" s="7" t="str">
         <x:v>否</x:v>
       </x:c>
-      <x:c r="Q17" s="7" t="str">
-        <x:v>通过</x:v>
-      </x:c>
-      <x:c r="R17" s="7" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="S17" s="7" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="T17" s="7" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="U17" s="7" t="str">
-        <x:v>passed</x:v>
-      </x:c>
-      <x:c r="V17" s="7" t="str">
-        <x:v>passed</x:v>
-      </x:c>
-      <x:c r="W17" s="7" t="str">
-        <x:v>raw/reports/final_176_01/public_accuracy.json#/cases/15</x:v>
+      <x:c r="Q17" s="7" t="inlineStr">
+        <x:is>
+          <x:t>通过</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="R17" s="7">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="S17" s="7">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="T17" s="7">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="U17" s="7" t="inlineStr">
+        <x:is>
+          <x:t>passed</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="V17" s="7" t="inlineStr">
+        <x:is>
+          <x:t>passed</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="W17" s="7" t="inlineStr">
+        <x:is>
+          <x:t>raw/reports/visible_page1g_final_accuracy.json#/cases/15</x:t>
+        </x:is>
       </x:c>
     </x:row>
     <x:row r="18" ht="30" customHeight="1">
@@ -3041,26 +3239,34 @@
       <x:c r="P18" s="7" t="str">
         <x:v>否</x:v>
       </x:c>
-      <x:c r="Q18" s="7" t="str">
-        <x:v>通过</x:v>
-      </x:c>
-      <x:c r="R18" s="7" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="S18" s="7" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="T18" s="7" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="U18" s="7" t="str">
-        <x:v>passed</x:v>
-      </x:c>
-      <x:c r="V18" s="7" t="str">
-        <x:v>passed</x:v>
-      </x:c>
-      <x:c r="W18" s="7" t="str">
-        <x:v>raw/reports/final_176_01/public_accuracy.json#/cases/16</x:v>
+      <x:c r="Q18" s="7" t="inlineStr">
+        <x:is>
+          <x:t>通过</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="R18" s="7">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="S18" s="7">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="T18" s="7">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="U18" s="7" t="inlineStr">
+        <x:is>
+          <x:t>passed</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="V18" s="7" t="inlineStr">
+        <x:is>
+          <x:t>passed</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="W18" s="7" t="inlineStr">
+        <x:is>
+          <x:t>raw/reports/visible_page1g_final_accuracy.json#/cases/16</x:t>
+        </x:is>
       </x:c>
     </x:row>
     <x:row r="19" ht="30" customHeight="1">
@@ -3112,26 +3318,34 @@
       <x:c r="P19" s="7" t="str">
         <x:v>否</x:v>
       </x:c>
-      <x:c r="Q19" s="7" t="str">
-        <x:v>通过</x:v>
-      </x:c>
-      <x:c r="R19" s="7" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="S19" s="7" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="T19" s="7" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="U19" s="7" t="str">
-        <x:v>passed</x:v>
-      </x:c>
-      <x:c r="V19" s="7" t="str">
-        <x:v>passed</x:v>
-      </x:c>
-      <x:c r="W19" s="7" t="str">
-        <x:v>raw/reports/final_176_01/public_accuracy.json#/cases/17</x:v>
+      <x:c r="Q19" s="7" t="inlineStr">
+        <x:is>
+          <x:t>通过</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="R19" s="7">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="S19" s="7">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="T19" s="7">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="U19" s="7" t="inlineStr">
+        <x:is>
+          <x:t>passed</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="V19" s="7" t="inlineStr">
+        <x:is>
+          <x:t>passed</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="W19" s="7" t="inlineStr">
+        <x:is>
+          <x:t>raw/reports/visible_page1g_final_accuracy.json#/cases/17</x:t>
+        </x:is>
       </x:c>
     </x:row>
     <x:row r="20" ht="30" customHeight="1">
@@ -3183,26 +3397,34 @@
       <x:c r="P20" s="7" t="str">
         <x:v>否</x:v>
       </x:c>
-      <x:c r="Q20" s="7" t="str">
-        <x:v>通过</x:v>
-      </x:c>
-      <x:c r="R20" s="7" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="S20" s="7" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="T20" s="7" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="U20" s="7" t="str">
-        <x:v>passed</x:v>
-      </x:c>
-      <x:c r="V20" s="7" t="str">
-        <x:v>passed</x:v>
-      </x:c>
-      <x:c r="W20" s="7" t="str">
-        <x:v>raw/reports/final_176_01/public_accuracy.json#/cases/18</x:v>
+      <x:c r="Q20" s="7" t="inlineStr">
+        <x:is>
+          <x:t>通过</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="R20" s="7">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="S20" s="7">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="T20" s="7">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="U20" s="7" t="inlineStr">
+        <x:is>
+          <x:t>passed</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="V20" s="7" t="inlineStr">
+        <x:is>
+          <x:t>passed</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="W20" s="7" t="inlineStr">
+        <x:is>
+          <x:t>raw/reports/visible_page1g_final_accuracy.json#/cases/18</x:t>
+        </x:is>
       </x:c>
     </x:row>
     <x:row r="21" ht="30" customHeight="1">
@@ -3254,26 +3476,34 @@
       <x:c r="P21" s="7" t="str">
         <x:v>否</x:v>
       </x:c>
-      <x:c r="Q21" s="7" t="str">
-        <x:v>通过</x:v>
-      </x:c>
-      <x:c r="R21" s="7" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="S21" s="7" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="T21" s="7" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="U21" s="7" t="str">
-        <x:v>passed</x:v>
-      </x:c>
-      <x:c r="V21" s="7" t="str">
-        <x:v>passed</x:v>
-      </x:c>
-      <x:c r="W21" s="7" t="str">
-        <x:v>raw/reports/final_176_01/public_accuracy.json#/cases/19</x:v>
+      <x:c r="Q21" s="7" t="inlineStr">
+        <x:is>
+          <x:t>通过</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="R21" s="7">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="S21" s="7">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="T21" s="7">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="U21" s="7" t="inlineStr">
+        <x:is>
+          <x:t>passed</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="V21" s="7" t="inlineStr">
+        <x:is>
+          <x:t>passed</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="W21" s="7" t="inlineStr">
+        <x:is>
+          <x:t>raw/reports/visible_page1g_final_accuracy.json#/cases/19</x:t>
+        </x:is>
       </x:c>
     </x:row>
     <x:row r="22" ht="30" customHeight="1">
@@ -3325,26 +3555,34 @@
       <x:c r="P22" s="7" t="str">
         <x:v>否</x:v>
       </x:c>
-      <x:c r="Q22" s="7" t="str">
-        <x:v>通过</x:v>
-      </x:c>
-      <x:c r="R22" s="7" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="S22" s="7" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="T22" s="7" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="U22" s="7" t="str">
-        <x:v>passed</x:v>
-      </x:c>
-      <x:c r="V22" s="7" t="str">
-        <x:v>passed</x:v>
-      </x:c>
-      <x:c r="W22" s="7" t="str">
-        <x:v>raw/reports/final_176_01/public_accuracy.json#/cases/20</x:v>
+      <x:c r="Q22" s="7" t="inlineStr">
+        <x:is>
+          <x:t>通过</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="R22" s="7">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="S22" s="7">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="T22" s="7">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="U22" s="7" t="inlineStr">
+        <x:is>
+          <x:t>passed</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="V22" s="7" t="inlineStr">
+        <x:is>
+          <x:t>passed</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="W22" s="7" t="inlineStr">
+        <x:is>
+          <x:t>raw/reports/visible_page1g_final_accuracy.json#/cases/20</x:t>
+        </x:is>
       </x:c>
     </x:row>
     <x:row r="23" ht="30" customHeight="1">
@@ -3396,26 +3634,34 @@
       <x:c r="P23" s="7" t="str">
         <x:v>否</x:v>
       </x:c>
-      <x:c r="Q23" s="7" t="str">
-        <x:v>通过</x:v>
-      </x:c>
-      <x:c r="R23" s="7" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="S23" s="7" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="T23" s="7" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="U23" s="7" t="str">
-        <x:v>passed</x:v>
-      </x:c>
-      <x:c r="V23" s="7" t="str">
-        <x:v>passed</x:v>
-      </x:c>
-      <x:c r="W23" s="7" t="str">
-        <x:v>raw/reports/final_176_01/public_accuracy.json#/cases/21</x:v>
+      <x:c r="Q23" s="7" t="inlineStr">
+        <x:is>
+          <x:t>通过</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="R23" s="7">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="S23" s="7">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="T23" s="7">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="U23" s="7" t="inlineStr">
+        <x:is>
+          <x:t>passed</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="V23" s="7" t="inlineStr">
+        <x:is>
+          <x:t>passed</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="W23" s="7" t="inlineStr">
+        <x:is>
+          <x:t>raw/reports/visible_page1g_final_accuracy.json#/cases/21</x:t>
+        </x:is>
       </x:c>
     </x:row>
     <x:row r="24" ht="30" customHeight="1">
@@ -3467,26 +3713,34 @@
       <x:c r="P24" s="7" t="str">
         <x:v>否</x:v>
       </x:c>
-      <x:c r="Q24" s="7" t="str">
-        <x:v>通过</x:v>
-      </x:c>
-      <x:c r="R24" s="7" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="S24" s="7" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="T24" s="7" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="U24" s="7" t="str">
-        <x:v>passed</x:v>
-      </x:c>
-      <x:c r="V24" s="7" t="str">
-        <x:v>passed</x:v>
-      </x:c>
-      <x:c r="W24" s="7" t="str">
-        <x:v>raw/reports/final_176_01/public_accuracy.json#/cases/22</x:v>
+      <x:c r="Q24" s="7" t="inlineStr">
+        <x:is>
+          <x:t>通过</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="R24" s="7">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="S24" s="7">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="T24" s="7">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="U24" s="7" t="inlineStr">
+        <x:is>
+          <x:t>passed</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="V24" s="7" t="inlineStr">
+        <x:is>
+          <x:t>passed</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="W24" s="7" t="inlineStr">
+        <x:is>
+          <x:t>raw/reports/visible_page1g_final_accuracy.json#/cases/22</x:t>
+        </x:is>
       </x:c>
     </x:row>
     <x:row r="25" ht="30" customHeight="1">
@@ -3538,26 +3792,34 @@
       <x:c r="P25" s="7" t="str">
         <x:v>否</x:v>
       </x:c>
-      <x:c r="Q25" s="7" t="str">
-        <x:v>通过</x:v>
-      </x:c>
-      <x:c r="R25" s="7" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="S25" s="7" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="T25" s="7" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="U25" s="7" t="str">
-        <x:v>passed</x:v>
-      </x:c>
-      <x:c r="V25" s="7" t="str">
-        <x:v>passed</x:v>
-      </x:c>
-      <x:c r="W25" s="7" t="str">
-        <x:v>raw/reports/final_176_01/public_accuracy.json#/cases/23</x:v>
+      <x:c r="Q25" s="7" t="inlineStr">
+        <x:is>
+          <x:t>通过</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="R25" s="7">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="S25" s="7">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="T25" s="7">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="U25" s="7" t="inlineStr">
+        <x:is>
+          <x:t>passed</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="V25" s="7" t="inlineStr">
+        <x:is>
+          <x:t>passed</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="W25" s="7" t="inlineStr">
+        <x:is>
+          <x:t>raw/reports/visible_page1g_final_accuracy.json#/cases/23</x:t>
+        </x:is>
       </x:c>
     </x:row>
     <x:row r="26" ht="30" customHeight="1">
@@ -3609,26 +3871,34 @@
       <x:c r="P26" s="7" t="str">
         <x:v>否</x:v>
       </x:c>
-      <x:c r="Q26" s="7" t="str">
-        <x:v>通过</x:v>
-      </x:c>
-      <x:c r="R26" s="7" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="S26" s="7" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="T26" s="7" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="U26" s="7" t="str">
-        <x:v>passed</x:v>
-      </x:c>
-      <x:c r="V26" s="7" t="str">
-        <x:v>passed</x:v>
-      </x:c>
-      <x:c r="W26" s="7" t="str">
-        <x:v>raw/reports/final_176_01/public_accuracy.json#/cases/24</x:v>
+      <x:c r="Q26" s="7" t="inlineStr">
+        <x:is>
+          <x:t>通过</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="R26" s="7">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="S26" s="7">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="T26" s="7">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="U26" s="7" t="inlineStr">
+        <x:is>
+          <x:t>passed</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="V26" s="7" t="inlineStr">
+        <x:is>
+          <x:t>passed</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="W26" s="7" t="inlineStr">
+        <x:is>
+          <x:t>raw/reports/visible_page1g_final_accuracy.json#/cases/24</x:t>
+        </x:is>
       </x:c>
     </x:row>
     <x:row r="27" ht="30" customHeight="1">
@@ -3680,26 +3950,34 @@
       <x:c r="P27" s="7" t="str">
         <x:v>否</x:v>
       </x:c>
-      <x:c r="Q27" s="7" t="str">
-        <x:v>通过</x:v>
-      </x:c>
-      <x:c r="R27" s="7" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="S27" s="7" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="T27" s="7" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="U27" s="7" t="str">
-        <x:v>passed</x:v>
-      </x:c>
-      <x:c r="V27" s="7" t="str">
-        <x:v>passed</x:v>
-      </x:c>
-      <x:c r="W27" s="7" t="str">
-        <x:v>raw/reports/final_176_01/public_accuracy.json#/cases/25</x:v>
+      <x:c r="Q27" s="7" t="inlineStr">
+        <x:is>
+          <x:t>通过</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="R27" s="7">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="S27" s="7">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="T27" s="7">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="U27" s="7" t="inlineStr">
+        <x:is>
+          <x:t>passed</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="V27" s="7" t="inlineStr">
+        <x:is>
+          <x:t>passed</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="W27" s="7" t="inlineStr">
+        <x:is>
+          <x:t>raw/reports/visible_page1g_final_accuracy.json#/cases/25</x:t>
+        </x:is>
       </x:c>
     </x:row>
     <x:row r="28" ht="30" customHeight="1">
@@ -3751,26 +4029,34 @@
       <x:c r="P28" s="7" t="str">
         <x:v>是</x:v>
       </x:c>
-      <x:c r="Q28" s="7" t="str">
-        <x:v>通过</x:v>
-      </x:c>
-      <x:c r="R28" s="7" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="S28" s="7" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="T28" s="7" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="U28" s="7" t="str">
-        <x:v>passed</x:v>
-      </x:c>
-      <x:c r="V28" s="7" t="str">
-        <x:v>passed</x:v>
-      </x:c>
-      <x:c r="W28" s="7" t="str">
-        <x:v>raw/reports/final_176_01/public_accuracy.json#/cases/26</x:v>
+      <x:c r="Q28" s="7" t="inlineStr">
+        <x:is>
+          <x:t>通过</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="R28" s="7">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="S28" s="7">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="T28" s="7">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="U28" s="7" t="inlineStr">
+        <x:is>
+          <x:t>passed</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="V28" s="7" t="inlineStr">
+        <x:is>
+          <x:t>passed</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="W28" s="7" t="inlineStr">
+        <x:is>
+          <x:t>raw/reports/visible_page1g_final_accuracy.json#/cases/26</x:t>
+        </x:is>
       </x:c>
     </x:row>
     <x:row r="29" ht="30" customHeight="1">
@@ -3822,26 +4108,34 @@
       <x:c r="P29" s="7" t="str">
         <x:v>是</x:v>
       </x:c>
-      <x:c r="Q29" s="7" t="str">
-        <x:v>通过</x:v>
-      </x:c>
-      <x:c r="R29" s="7" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="S29" s="7" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="T29" s="7" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="U29" s="7" t="str">
-        <x:v>passed</x:v>
-      </x:c>
-      <x:c r="V29" s="7" t="str">
-        <x:v>passed</x:v>
-      </x:c>
-      <x:c r="W29" s="7" t="str">
-        <x:v>raw/reports/final_176_01/public_accuracy.json#/cases/27</x:v>
+      <x:c r="Q29" s="7" t="inlineStr">
+        <x:is>
+          <x:t>通过</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="R29" s="7">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="S29" s="7">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="T29" s="7">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="U29" s="7" t="inlineStr">
+        <x:is>
+          <x:t>passed</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="V29" s="7" t="inlineStr">
+        <x:is>
+          <x:t>passed</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="W29" s="7" t="inlineStr">
+        <x:is>
+          <x:t>raw/reports/visible_page1g_final_accuracy.json#/cases/27</x:t>
+        </x:is>
       </x:c>
     </x:row>
     <x:row r="30" ht="30" customHeight="1">
@@ -3893,26 +4187,34 @@
       <x:c r="P30" s="7" t="str">
         <x:v>是</x:v>
       </x:c>
-      <x:c r="Q30" s="7" t="str">
-        <x:v>通过</x:v>
-      </x:c>
-      <x:c r="R30" s="7" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="S30" s="7" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="T30" s="7" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="U30" s="7" t="str">
-        <x:v>passed</x:v>
-      </x:c>
-      <x:c r="V30" s="7" t="str">
-        <x:v>passed</x:v>
-      </x:c>
-      <x:c r="W30" s="7" t="str">
-        <x:v>raw/reports/final_176_01/public_accuracy.json#/cases/28</x:v>
+      <x:c r="Q30" s="7" t="inlineStr">
+        <x:is>
+          <x:t>通过</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="R30" s="7">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="S30" s="7">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="T30" s="7">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="U30" s="7" t="inlineStr">
+        <x:is>
+          <x:t>passed</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="V30" s="7" t="inlineStr">
+        <x:is>
+          <x:t>passed</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="W30" s="7" t="inlineStr">
+        <x:is>
+          <x:t>raw/reports/visible_page1g_final_accuracy.json#/cases/28</x:t>
+        </x:is>
       </x:c>
     </x:row>
     <x:row r="31" ht="30" customHeight="1">
@@ -3964,26 +4266,34 @@
       <x:c r="P31" s="7" t="str">
         <x:v>是</x:v>
       </x:c>
-      <x:c r="Q31" s="7" t="str">
-        <x:v>通过</x:v>
-      </x:c>
-      <x:c r="R31" s="7" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="S31" s="7" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="T31" s="7" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="U31" s="7" t="str">
-        <x:v>passed</x:v>
-      </x:c>
-      <x:c r="V31" s="7" t="str">
-        <x:v>passed</x:v>
-      </x:c>
-      <x:c r="W31" s="7" t="str">
-        <x:v>raw/reports/final_176_01/public_accuracy.json#/cases/29</x:v>
+      <x:c r="Q31" s="7" t="inlineStr">
+        <x:is>
+          <x:t>通过</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="R31" s="7">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="S31" s="7">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="T31" s="7">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="U31" s="7" t="inlineStr">
+        <x:is>
+          <x:t>passed</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="V31" s="7" t="inlineStr">
+        <x:is>
+          <x:t>passed</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="W31" s="7" t="inlineStr">
+        <x:is>
+          <x:t>raw/reports/visible_page1g_final_accuracy.json#/cases/29</x:t>
+        </x:is>
       </x:c>
     </x:row>
     <x:row r="32" ht="30" customHeight="1">
@@ -4035,26 +4345,34 @@
       <x:c r="P32" s="7" t="str">
         <x:v>是</x:v>
       </x:c>
-      <x:c r="Q32" s="7" t="str">
-        <x:v>通过</x:v>
-      </x:c>
-      <x:c r="R32" s="7" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="S32" s="7" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="T32" s="7" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="U32" s="7" t="str">
-        <x:v>passed</x:v>
-      </x:c>
-      <x:c r="V32" s="7" t="str">
-        <x:v>passed</x:v>
-      </x:c>
-      <x:c r="W32" s="7" t="str">
-        <x:v>raw/reports/final_176_01/public_accuracy.json#/cases/30</x:v>
+      <x:c r="Q32" s="7" t="inlineStr">
+        <x:is>
+          <x:t>通过</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="R32" s="7">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="S32" s="7">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="T32" s="7">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="U32" s="7" t="inlineStr">
+        <x:is>
+          <x:t>passed</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="V32" s="7" t="inlineStr">
+        <x:is>
+          <x:t>passed</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="W32" s="7" t="inlineStr">
+        <x:is>
+          <x:t>raw/reports/visible_page1g_final_accuracy.json#/cases/30</x:t>
+        </x:is>
       </x:c>
     </x:row>
     <x:row r="33" ht="30" customHeight="1">
@@ -4106,26 +4424,34 @@
       <x:c r="P33" s="7" t="str">
         <x:v>是</x:v>
       </x:c>
-      <x:c r="Q33" s="7" t="str">
-        <x:v>通过</x:v>
-      </x:c>
-      <x:c r="R33" s="7" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="S33" s="7" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="T33" s="7" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="U33" s="7" t="str">
-        <x:v>passed</x:v>
-      </x:c>
-      <x:c r="V33" s="7" t="str">
-        <x:v>passed</x:v>
-      </x:c>
-      <x:c r="W33" s="7" t="str">
-        <x:v>raw/reports/final_176_01/public_accuracy.json#/cases/31</x:v>
+      <x:c r="Q33" s="7" t="inlineStr">
+        <x:is>
+          <x:t>通过</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="R33" s="7">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="S33" s="7">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="T33" s="7">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="U33" s="7" t="inlineStr">
+        <x:is>
+          <x:t>passed</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="V33" s="7" t="inlineStr">
+        <x:is>
+          <x:t>passed</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="W33" s="7" t="inlineStr">
+        <x:is>
+          <x:t>raw/reports/visible_page1g_final_accuracy.json#/cases/31</x:t>
+        </x:is>
       </x:c>
     </x:row>
     <x:row r="34" ht="30" customHeight="1">
@@ -4177,26 +4503,34 @@
       <x:c r="P34" s="7" t="str">
         <x:v>是</x:v>
       </x:c>
-      <x:c r="Q34" s="7" t="str">
-        <x:v>通过</x:v>
-      </x:c>
-      <x:c r="R34" s="7" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="S34" s="7" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="T34" s="7" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="U34" s="7" t="str">
-        <x:v>passed</x:v>
-      </x:c>
-      <x:c r="V34" s="7" t="str">
-        <x:v>passed</x:v>
-      </x:c>
-      <x:c r="W34" s="7" t="str">
-        <x:v>raw/reports/final_176_01/public_accuracy.json#/cases/32</x:v>
+      <x:c r="Q34" s="7" t="inlineStr">
+        <x:is>
+          <x:t>通过</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="R34" s="7">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="S34" s="7">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="T34" s="7">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="U34" s="7" t="inlineStr">
+        <x:is>
+          <x:t>passed</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="V34" s="7" t="inlineStr">
+        <x:is>
+          <x:t>passed</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="W34" s="7" t="inlineStr">
+        <x:is>
+          <x:t>raw/reports/visible_page1g_final_accuracy.json#/cases/32</x:t>
+        </x:is>
       </x:c>
     </x:row>
     <x:row r="35" ht="30" customHeight="1">
@@ -4248,26 +4582,34 @@
       <x:c r="P35" s="7" t="str">
         <x:v>是</x:v>
       </x:c>
-      <x:c r="Q35" s="7" t="str">
-        <x:v>通过</x:v>
-      </x:c>
-      <x:c r="R35" s="7" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="S35" s="7" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="T35" s="7" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="U35" s="7" t="str">
-        <x:v>passed</x:v>
-      </x:c>
-      <x:c r="V35" s="7" t="str">
-        <x:v>passed</x:v>
-      </x:c>
-      <x:c r="W35" s="7" t="str">
-        <x:v>raw/reports/final_176_01/public_accuracy.json#/cases/33</x:v>
+      <x:c r="Q35" s="7" t="inlineStr">
+        <x:is>
+          <x:t>通过</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="R35" s="7">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="S35" s="7">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="T35" s="7">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="U35" s="7" t="inlineStr">
+        <x:is>
+          <x:t>passed</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="V35" s="7" t="inlineStr">
+        <x:is>
+          <x:t>passed</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="W35" s="7" t="inlineStr">
+        <x:is>
+          <x:t>raw/reports/visible_page1g_final_accuracy.json#/cases/33</x:t>
+        </x:is>
       </x:c>
     </x:row>
     <x:row r="36" ht="30" customHeight="1">
@@ -4319,26 +4661,34 @@
       <x:c r="P36" s="7" t="str">
         <x:v>是</x:v>
       </x:c>
-      <x:c r="Q36" s="7" t="str">
-        <x:v>通过</x:v>
-      </x:c>
-      <x:c r="R36" s="7" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="S36" s="7" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="T36" s="7" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="U36" s="7" t="str">
-        <x:v>passed</x:v>
-      </x:c>
-      <x:c r="V36" s="7" t="str">
-        <x:v>passed</x:v>
-      </x:c>
-      <x:c r="W36" s="7" t="str">
-        <x:v>raw/reports/final_176_01/public_accuracy.json#/cases/34</x:v>
+      <x:c r="Q36" s="7" t="inlineStr">
+        <x:is>
+          <x:t>通过</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="R36" s="7">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="S36" s="7">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="T36" s="7">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="U36" s="7" t="inlineStr">
+        <x:is>
+          <x:t>passed</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="V36" s="7" t="inlineStr">
+        <x:is>
+          <x:t>passed</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="W36" s="7" t="inlineStr">
+        <x:is>
+          <x:t>raw/reports/visible_page1g_final_accuracy.json#/cases/34</x:t>
+        </x:is>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>